<commit_message>
Updated loggers and Environment in Fixed test cases
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (10).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (10).xlsx
@@ -538,7 +538,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TestSigma_06-03-2026_SC1_C4_411</v>
+        <v>TestSigma_09-03-2026_SC1_MV_297</v>
       </c>
       <c r="B2">
         <v>2001</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TestSigma_06-03-2026_SC1_0F_473</v>
+        <v>TestSigma_09-03-2026_SC1_72_589</v>
       </c>
       <c r="B3">
         <v>2001</v>

</xml_diff>

<commit_message>
fixed Bidmap testcases including locators, prereqs and stepgroups
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (10).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (10).xlsx
@@ -538,7 +538,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TestSigma_09-03-2026_SC1_MV_297</v>
+        <v>TestSigma_09-03-2026_SC1_VC_385</v>
       </c>
       <c r="B2">
         <v>2001</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TestSigma_09-03-2026_SC1_72_589</v>
+        <v>TestSigma_09-03-2026_SC1_K8_534</v>
       </c>
       <c r="B3">
         <v>2001</v>

</xml_diff>

<commit_message>
commiting changes-4 scripts-1PreReq-minor changes in index.ts,elements,tdp
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (10).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (10).xlsx
@@ -538,7 +538,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TestSigma_09-03-2026_SC1_VC_385</v>
+        <v>TestSigma_12-03-2026_SC1_3M_631</v>
       </c>
       <c r="B2">
         <v>2001</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TestSigma_09-03-2026_SC1_K8_534</v>
+        <v>TestSigma_12-03-2026_SC1_EK_199</v>
       </c>
       <c r="B3">
         <v>2001</v>

</xml_diff>

<commit_message>
Commiting the changes of updated scripts-Reworked on Pre-reqs,implemented loggers and remove tdp from step group level
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (10).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (10).xlsx
@@ -538,7 +538,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TestSigma_12-03-2026_SC1_3M_631</v>
+        <v>TestSigma_13-03-2026_SC1_8X_859</v>
       </c>
       <c r="B2">
         <v>2001</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TestSigma_12-03-2026_SC1_EK_199</v>
+        <v>TestSigma_13-03-2026_SC1_0K_944</v>
       </c>
       <c r="B3">
         <v>2001</v>

</xml_diff>